<commit_message>
remap_tf_noise_gsea: regenerate with current data, composite and PDFs
- AUC significance as in ruido_summary (Wald with DeLong variance, BH):
  514 consistent TFs, all low noise
- GSEA with fixed seed; panel B highlights MLL1/2 complex (GO:0044665),
  significant in both replicates (MLL1 complex only in Rep 1)
- composite remap_tf_noise_gsea (A AUC, B GSEA), JPG and PDF

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figures/R3.7_remap_tf_noise_gsea/GSEA_remap_noise.xlsx
+++ b/figures/R3.7_remap_tf_noise_gsea/GSEA_remap_noise.xlsx
@@ -352,7 +352,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -415,989 +415,817 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GO:0005856</t>
+          <t>GO:0000785</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>cytoskeleton</t>
+          <t>chromatin</t>
         </is>
       </c>
       <c r="C2">
-        <v>69</v>
+        <v>476</v>
       </c>
       <c r="D2">
-        <v>-0.1694407540093076</v>
+        <v>-0.1909552710171361</v>
       </c>
       <c r="E2">
-        <v>-1.706511489926708</v>
+        <v>-3.912097189036784</v>
       </c>
       <c r="F2">
-        <v>0.01499209166741207</v>
+        <v>5.037466448099576E-10</v>
       </c>
       <c r="G2">
-        <v>0.08413827657748955</v>
+        <v>5.793086415314513E-08</v>
       </c>
       <c r="H2">
-        <v>0.06700256349877887</v>
+        <v>4.666284709818555E-08</v>
       </c>
       <c r="I2">
-        <v>434</v>
+        <v>362</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>tags=62%, list=45%, signal=37%</t>
+          <t>tags=49%, list=38%, signal=60%</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>7756/79692/11083/60436/2101/1499/9611/10735/84307/29855/6907/324/6714/3190/5324/9112/2648/7157/79718/1877/11091/8243/10856/3183/5885/4089/54617/6497/9314/672/9584/7029/1021/3297/5977/5914/10274/9126/10951/2908/5925/4780/1869</t>
+          <t>83855/55249/84148/571/3190/147912/2305/9839/6657/2118/23764/1523/367/9611/5309/2627/3726/1105/7392/2355/1386/60436/2115/5090/28999/10608/7080/8626/1051/79977/5316/9112/51548/3169/4286/57178/6777/10445/11278/56970/4609/55553/221037/11016/5927/3170/7027/10919/23030/54617/10042/3183/8473/23476/408/2626/55145/26205/3200/11091/7544/6886/9219/6688/3662/7157/9188/56980/7913/51230/11244/3110/116113/7543/55818/7022/5885/2002/10856/3660/57504/6495/121340/5993/8861/860/5468/221937/10725/2353/6929/22882/23081/2623/2145/7182/5970/1050/4772/2648/23309/7004/1406/5469/23435/4205/6945/6935/9314/4802/9889/2308/9324/6928/30009/7030/8289/3066/79923/4089/7029/93986/6598/23512/64843/7421/6774/1052/1316/8932/11279/2313/466/9070/546/2146/5977/4335/2551/3172/2033/26959/4790/7071/7391/9126/467/25836/27086/10274/6909/3659/3297/196/6722/23269/6096/4654/4086/5914/389058/6934/2908/8553/6045/4801/27125/23028/5079/2625/5451/10951/64919/3054/1387/6670/6599/10691/4090/53335/5925/4778/3065/5241/4760/6938/4780/10481/1390/2113/1958/6772/3725/4094/8805/3091/10661/3727/3516/2078/4088/4209/8019/688/196528/861/65980/10215/4601/9682/687/1106/1876/25942/4800/4149/1874/6671/4613/1997/7528/7936/405/10765/1869/1385/6668/6872/6667/6046/6908</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GO:0034708</t>
+          <t>GO:0032991</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>methyltransferase complex</t>
+          <t>protein-containing complex</t>
         </is>
       </c>
       <c r="C3">
-        <v>36</v>
+        <v>428</v>
       </c>
       <c r="D3">
-        <v>-0.2432758509903516</v>
+        <v>-0.1906661663610363</v>
       </c>
       <c r="E3">
-        <v>-1.814747423677504</v>
+        <v>-3.7913930898397</v>
       </c>
       <c r="F3">
-        <v>0.01889676101685396</v>
+        <v>1.446707341098378E-09</v>
       </c>
       <c r="G3">
-        <v>0.0944838050842698</v>
+        <v>8.318567211315675E-08</v>
       </c>
       <c r="H3">
-        <v>0.07524110793896086</v>
+        <v>6.700539264034594E-08</v>
       </c>
       <c r="I3">
-        <v>209</v>
+        <v>361</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>tags=47%, list=22%, signal=38%</t>
+          <t>tags=50%, list=38%, signal=56%</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>51230/11091/10856/8085/23512/3066/4297/23269/2146/9070/3054/6045/5929/9757/1876/4149/6872</t>
+          <t>55249/84148/571/3190/147912/7307/6657/23764/367/9611/2627/3726/2355/1386/171023/5090/10153/7080/8626/1051/324/4298/5316/6907/9112/602/4286/6426/10614/6777/10445/56970/4609/221037/11016/5927/26523/7027/132660/657/54617/10042/3183/8473/4683/22976/2626/3609/11091/6886/9219/81608/6688/3662/7157/9188/56980/7913/7538/51230/80816/55818/8314/5885/8243/10856/57504/6495/5993/8861/860/5468/10725/83860/7520/2353/6929/9968/7494/2623/2145/79718/5970/1050/4772/2648/23309/7004/1406/5469/22936/4205/8085/10589/5093/9314/9584/4802/4605/6928/7764/6497/8289/3066/84844/4089/7029/6598/23512/7421/6774/1052/8932/905/466/4297/5994/9070/1487/2146/5977/2033/672/4790/1021/7391/9126/51497/467/25836/10274/6909/3297/196/23269/23186/4654/4086/5914/6934/2908/6045/4801/27125/23028/5451/92906/64919/5929/3054/1387/2624/6670/55726/6599/4841/51341/4090/53335/5925/4778/3065/4760/4686/1022/6938/4780/10481/1027/4851/1390/2962/6772/3725/4094/3091/2959/4602/3727/54973/3516/8328/2078/4088/688/1024/196528/9757/861/65980/4601/1876/25942/4800/54880/865/4149/1874/5978/9441/6829/5460/7528/7936/405/1025/1869/1385/6872/6667/7469/6908</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GO:0035097</t>
+          <t>GO:0140513</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>histone methyltransferase complex</t>
+          <t>nuclear protein-containing complex</t>
         </is>
       </c>
       <c r="C4">
-        <v>36</v>
+        <v>287</v>
       </c>
       <c r="D4">
-        <v>-0.2432758509903516</v>
+        <v>-0.1918911901228944</v>
       </c>
       <c r="E4">
-        <v>-1.814747423677504</v>
+        <v>-3.388039789732365</v>
       </c>
       <c r="F4">
-        <v>0.01889676101685396</v>
+        <v>5.451642128031299E-08</v>
       </c>
       <c r="G4">
-        <v>0.0944838050842698</v>
+        <v>2.089796149078665E-06</v>
       </c>
       <c r="H4">
-        <v>0.07524110793896086</v>
+        <v>1.683314060585103E-06</v>
       </c>
       <c r="I4">
-        <v>209</v>
+        <v>302</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>tags=47%, list=22%, signal=38%</t>
+          <t>tags=47%, list=31%, signal=46%</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>51230/11091/10856/8085/23512/3066/4297/23269/2146/9070/3054/6045/5929/9757/1876/4149/6872</t>
+          <t>10614/6777/10445/56970/4609/221037/11016/7027/132660/54617/10042/3183/8473/4683/22976/2626/11091/9219/81608/9188/7913/51230/80816/55818/8314/10856/57504/5993/8861/5468/83860/7520/2353/6929/9968/7494/2145/79718/5970/1050/2648/23309/1406/5469/22936/8085/10589/4802/4605/7764/8289/3066/84844/4089/7029/6598/23512/7421/6774/1052/8932/905/466/4297/5994/9070/2146/5977/672/4790/51497/467/25836/196/23269/23186/4086/5914/6934/6045/4801/27125/5451/64919/5929/3054/55726/6599/4841/51341/4090/53335/5925/4778/3065/4760/1022/6938/4780/1390/2962/6772/3725/4094/3091/2959/4602/3727/54973/4088/1024/196528/9757/861/65980/4601/1876/25942/4800/54880/865/4149/1874/9441/6829/7528/7936/405/1025/1869/1385/6872/7469/6908</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GO:0016514</t>
+          <t>GO:0005667</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SWI/SNF complex</t>
+          <t>transcription regulator complex</t>
         </is>
       </c>
       <c r="C5">
-        <v>17</v>
+        <v>234</v>
       </c>
       <c r="D5">
-        <v>-0.3612059375162823</v>
+        <v>-0.2000512206295649</v>
       </c>
       <c r="E5">
-        <v>-1.846547262710934</v>
+        <v>-3.397431211830044</v>
       </c>
       <c r="F5">
-        <v>0.01422517643897774</v>
+        <v>1.890659181794096E-07</v>
       </c>
       <c r="G5">
-        <v>0.08413827657748955</v>
+        <v>5.435645147658025E-06</v>
       </c>
       <c r="H5">
-        <v>0.06700256349877887</v>
+        <v>4.378368631523169E-06</v>
       </c>
       <c r="I5">
-        <v>144</v>
+        <v>223</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>tags=53%, list=15%, signal=46%</t>
+          <t>tags=40%, list=23%, signal=41%</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>8289/5977/6598/64919/5925/53335/6599/65980/196528</t>
+          <t>57504/6495/5993/8861/860/5468/10725/83860/2353/6929/7494/2623/79718/5970/1050/4772/2648/7004/1406/5469/4205/10589/9314/4802/6928/6497/3066/4089/7029/7421/6774/1052/8932/466/5994/1487/2033/4790/7391/467/6909/196/23186/4654/4086/5914/6934/4801/23028/5451/1387/2624/6670/4841/4090/5925/4778/3065/4760/1022/6938/4780/10481/1390/2962/6772/3725/4094/3091/2959/4602/3727/3516/8328/4088/688/861/4601/1876/25942/4800/865/4149/1874/5978/9441/5460/7528/405/1869/1385/6872/6667/6908</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GO:0032993</t>
+          <t>GO:0090575</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>protein-DNA complex</t>
+          <t>RNA polymerase II transcription regulator complex</t>
         </is>
       </c>
       <c r="C6">
-        <v>37</v>
+        <v>122</v>
       </c>
       <c r="D6">
-        <v>-0.245948943153591</v>
+        <v>-0.2467069906227108</v>
       </c>
       <c r="E6">
-        <v>-1.855632546043184</v>
+        <v>-3.187831821825059</v>
       </c>
       <c r="F6">
-        <v>0.01536438094023722</v>
+        <v>7.620835687320805E-07</v>
       </c>
       <c r="G6">
-        <v>0.08413827657748955</v>
+        <v>1.752792208083785E-05</v>
       </c>
       <c r="H6">
-        <v>0.06700256349877887</v>
+        <v>1.41186008522996E-05</v>
       </c>
       <c r="I6">
-        <v>244</v>
+        <v>219</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>tags=51%, list=25%, signal=40%</t>
+          <t>tags=47%, list=23%, signal=41%</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2623/3662/2353/7520/4802/10856/7004/5469/23512/4801/4778/2033/6934/6670/4780/2959/4800/4149/6667</t>
+          <t>5993/8861/5468/83860/2353/6929/7494/1050/2648/1406/5469/10589/4802/4089/7029/7421/6774/1052/466/5994/467/4086/5914/6934/4801/5451/4841/4090/5925/4778/4760/1022/6938/4780/1390/2962/6772/3725/4094/3091/2959/4602/3727/4088/861/4601/1876/4800/865/4149/1874/9441/405/1869/1385/6872/6908</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GO:0036464</t>
+          <t>GO:0005737</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>cytoplasmic ribonucleoprotein granule</t>
+          <t>cytoplasm</t>
         </is>
       </c>
       <c r="C7">
-        <v>11</v>
+        <v>424</v>
       </c>
       <c r="D7">
-        <v>-0.4700944386149003</v>
+        <v>-0.1307246617692976</v>
       </c>
       <c r="E7">
-        <v>-1.903597354560582</v>
+        <v>-2.607176968439508</v>
       </c>
       <c r="F7">
-        <v>0.01324271621020897</v>
+        <v>7.604927659906119E-05</v>
       </c>
       <c r="G7">
-        <v>0.08413827657748955</v>
+        <v>0.00145761113481534</v>
       </c>
       <c r="H7">
-        <v>0.06700256349877887</v>
+        <v>0.001174094094862699</v>
       </c>
       <c r="I7">
-        <v>517</v>
+        <v>427</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>tags=100%, list=54%, signal=47%</t>
+          <t>tags=53%, list=44%, signal=53%</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2553/9575/3190/7538/7706/26523/64332/23435/5093/1025</t>
+          <t>90850/5928/2553/11083/1499/22880/4824/6879/6591/7023/3191/3146/2099/6498/55929/3215/2077/4901/9575/58517/7706/2122/5458/64344/2101/7750/23429/79692/5948/90993/10782/3661/57591/3651/2521/3096/55249/84148/571/3190/147912/51523/9839/6657/23764/1523/367/9611/1105/1386/8626/5324/1051/324/4298/5316/9112/602/51548/7026/4286/6426/84662/7541/10614/57178/6777/10445/11278/7775/4609/55553/8148/11016/3170/26523/7027/54617/3183/8473/49854/4683/408/26205/3609/81608/3662/7157/9188/7913/7538/51230/3110/55818/1820/8314/7022/5885/2002/8243/10856/3660/64332/57504/6495/7728/121340/860/5468/221937/10725/7520/2353/6929/22882/7494/5970/4772/1877/2648/23309/7004/23435/4205/6945/6935/5093/9314/9889/4605/2308/9324/7764/7030/6497/3066/4089/7421/6774/1316/8932/11279/905/2313/4297/1487/5977/3172/2033/672/4790/140690/1021/7391/9126/25836/10274/6909/3659/3297/196/6722/55734/4654/4086/5914/2908/8553/6045/5451/80319/3054/1387/2624/6670/55726/604/6599/10691/51341/5371/4090/53335/5925/4778/3065/5241/4760/4686/1022/6938/4780/1027/4851/1390/2113/1958/6772/4094/8805/3091/4602/54973/3516/2078/4088/4899/4209/688/10215/4601/9682/687/1874/6671/5978/5460/405/1025/10765/1869/6667/7469/6046/6908</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GO:0035770</t>
+          <t>GO:0061695</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ribonucleoprotein granule</t>
+          <t>transferase complex, transferring phosphorus-containing groups</t>
         </is>
       </c>
       <c r="C8">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="D8">
-        <v>-0.4710830704521556</v>
+        <v>-0.4194549442984999</v>
       </c>
       <c r="E8">
-        <v>-2.09141312499695</v>
+        <v>-2.571983965194609</v>
       </c>
       <c r="F8">
-        <v>0.003576926588493112</v>
+        <v>0.0002959107113133732</v>
       </c>
       <c r="G8">
-        <v>0.02570915985479424</v>
+        <v>0.003993774280120856</v>
       </c>
       <c r="H8">
-        <v>0.02047319823676979</v>
+        <v>0.003216953195886822</v>
       </c>
       <c r="I8">
-        <v>517</v>
+        <v>209</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>tags=100%, list=54%, signal=47%</t>
+          <t>tags=65%, list=22%, signal=52%</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>3191/2553/9575/3190/7538/7706/26523/64332/23435/5093/3297/1025</t>
+          <t>83860/7520/9968/2648/905/1021/51341/5925/1022/2962/2959/1024/1025/6872/6908</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GO:1990234</t>
+          <t>GO:1902554</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>transferase complex</t>
+          <t>serine/threonine protein kinase complex</t>
         </is>
       </c>
       <c r="C9">
-        <v>81</v>
+        <v>11</v>
       </c>
       <c r="D9">
-        <v>-0.1981038861468934</v>
+        <v>-0.5930217256818234</v>
       </c>
       <c r="E9">
-        <v>-2.160269231116381</v>
+        <v>-2.460202052552936</v>
       </c>
       <c r="F9">
-        <v>0.004850524774398883</v>
+        <v>0.0003125562480094583</v>
       </c>
       <c r="G9">
-        <v>0.03281237347387479</v>
+        <v>0.003993774280120856</v>
       </c>
       <c r="H9">
-        <v>0.02612976194258222</v>
+        <v>0.003216953195886822</v>
       </c>
       <c r="I9">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>tags=42%, list=22%, signal=36%</t>
+          <t>tags=82%, list=22%, signal=65%</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>51230/11091/10856/5469/8085/83860/672/23512/1021/3066/4297/23269/905/2146/9070/2033/3054/1022/1027/1387/6045/5925/2962/2959/5929/51341/1024/9757/1876/54880/1025/4149/6908/6872</t>
+          <t>7520/9968/905/1021/51341/5925/1022/1024/1025</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GO:0061695</t>
+          <t>GO:1902911</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>transferase complex, transferring phosphorus-containing groups</t>
+          <t>protein kinase complex</t>
         </is>
       </c>
       <c r="C10">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="D10">
-        <v>-0.370576864866505</v>
+        <v>-0.5930217256818234</v>
       </c>
       <c r="E10">
-        <v>-2.203271392255046</v>
+        <v>-2.460202052552936</v>
       </c>
       <c r="F10">
-        <v>0.001750055033476567</v>
+        <v>0.0003125562480094583</v>
       </c>
       <c r="G10">
-        <v>0.01341708858998701</v>
+        <v>0.003993774280120856</v>
       </c>
       <c r="H10">
-        <v>0.01068454652017272</v>
+        <v>0.003216953195886822</v>
       </c>
       <c r="I10">
-        <v>299</v>
+        <v>208</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>tags=70%, list=31%, signal=49%</t>
+          <t>tags=82%, list=22%, signal=65%</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>56970/2648/9968/7520/83860/1021/905/1022/5925/2962/2959/51341/1024/1025/6908/6872</t>
+          <t>7520/9968/905/1021/51341/5925/1022/1024/1025</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GO:0099080</t>
+          <t>GO:0044665</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>supramolecular complex</t>
+          <t>MLL1/2 complex</t>
         </is>
       </c>
       <c r="C11">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="D11">
-        <v>-0.2977691607928926</v>
+        <v>-0.4569606801275239</v>
       </c>
       <c r="E11">
-        <v>-2.246605083520115</v>
+        <v>-2.470144736835616</v>
       </c>
       <c r="F11">
-        <v>0.001633792763539584</v>
+        <v>0.0004025729741143032</v>
       </c>
       <c r="G11">
-        <v>0.01341708858998701</v>
+        <v>0.004629589202314486</v>
       </c>
       <c r="H11">
-        <v>0.01068454652017272</v>
+        <v>0.003729097023374598</v>
       </c>
       <c r="I11">
-        <v>441</v>
+        <v>531</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>tags=76%, list=46%, signal=43%</t>
+          <t>tags=100%, list=55%, signal=46%</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2553/7756/9575/1499/6597/23468/324/6714/3190/9112/7913/7538/7706/26523/92822/64332/8243/23435/5093/54617/3297/6598/4654/2959/6599/196528/25942/1025</t>
+          <t>4221/57680/6879/84148/10445/11091/51230/10856/4297/9070/23269/6045/5929/3054/9757/1876/4149/6872</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GO:1902554</t>
+          <t>GO:0099080</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>serine/threonine protein kinase complex</t>
+          <t>supramolecular complex</t>
         </is>
       </c>
       <c r="C12">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="D12">
-        <v>-0.5568722512601556</v>
+        <v>-0.3174749497148329</v>
       </c>
       <c r="E12">
-        <v>-2.254994863267092</v>
+        <v>-2.376005076063928</v>
       </c>
       <c r="F12">
-        <v>0.001567094756395386</v>
+        <v>0.0004763600854654198</v>
       </c>
       <c r="G12">
-        <v>0.01341708858998701</v>
+        <v>0.004980128166229389</v>
       </c>
       <c r="H12">
-        <v>0.01068454652017272</v>
+        <v>0.004011453351287745</v>
       </c>
       <c r="I12">
-        <v>246</v>
+        <v>473</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>tags=82%, list=26%, signal=62%</t>
+          <t>tags=81%, list=49%, signal=43%</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>9968/7520/1021/905/1022/5925/51341/1024/1025</t>
+          <t>23468/6714/7756/6597/2553/1499/3191/9575/7706/84148/3190/324/9112/26523/54617/7913/7538/92822/8243/64332/23435/5093/6598/3297/4654/6599/2959/196528/25942/1025</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GO:1902911</t>
+          <t>GO:0071339</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>protein kinase complex</t>
+          <t>MLL1 complex</t>
         </is>
       </c>
       <c r="C13">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D13">
-        <v>-0.5568722512601556</v>
+        <v>-0.4564755838641189</v>
       </c>
       <c r="E13">
-        <v>-2.254994863267092</v>
+        <v>-2.368974252099638</v>
       </c>
       <c r="F13">
-        <v>0.001567094756395386</v>
+        <v>0.0005456648076065526</v>
       </c>
       <c r="G13">
-        <v>0.01341708858998701</v>
+        <v>0.005229287739562796</v>
       </c>
       <c r="H13">
-        <v>0.01068454652017272</v>
+        <v>0.004212149392050581</v>
       </c>
       <c r="I13">
-        <v>246</v>
+        <v>531</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>tags=82%, list=26%, signal=62%</t>
+          <t>tags=100%, list=55%, signal=46%</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>9968/7520/1021/905/1022/5925/51341/1024/1025</t>
+          <t>4221/57680/6879/84148/10445/11091/51230/10856/4297/9070/23269/6045/5929/3054/1876/4149/6872</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GO:0000791</t>
+          <t>GO:1902494</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>euchromatin</t>
+          <t>catalytic complex</t>
         </is>
       </c>
       <c r="C14">
-        <v>23</v>
+        <v>148</v>
       </c>
       <c r="D14">
-        <v>-0.3808713614105275</v>
+        <v>-0.1632131114967814</v>
       </c>
       <c r="E14">
-        <v>-2.264477505975296</v>
+        <v>-2.290977009638185</v>
       </c>
       <c r="F14">
-        <v>0.001162949997651638</v>
+        <v>0.000738025321725288</v>
       </c>
       <c r="G14">
-        <v>0.01215811361181258</v>
+        <v>0.006062350857029151</v>
       </c>
       <c r="H14">
-        <v>0.009681976057004067</v>
+        <v>0.004883175061039501</v>
       </c>
       <c r="I14">
-        <v>202</v>
+        <v>321</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>tags=61%, list=21%, signal=49%</t>
+          <t>tags=49%, list=33%, signal=39%</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>10856/6929/9314/3297/9070/27125/4654/6045/3725/3091/8805/6667/1385/6908</t>
+          <t>324/6907/9112/6426/10445/56970/221037/26523/54617/10042/3183/8473/22976/11091/9219/9188/7913/51230/55818/10856/57504/83860/7520/9968/2145/79718/2648/23309/5469/8085/7764/8289/3066/6598/23512/8932/905/4297/9070/2146/5977/2033/672/1021/23269/23186/6045/23028/64919/5929/3054/1387/6599/51341/53335/5925/3065/1022/1027/2962/2959/1024/196528/9757/65980/1876/25942/54880/4149/7528/1025/6872/6908</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GO:0071339</t>
+          <t>GO:0005829</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MLL1 complex</t>
+          <t>cytosol</t>
         </is>
       </c>
       <c r="C15">
-        <v>18</v>
+        <v>249</v>
       </c>
       <c r="D15">
-        <v>-0.440968698762612</v>
+        <v>-0.1323209941308882</v>
       </c>
       <c r="E15">
-        <v>-2.30863671650667</v>
+        <v>-2.270186400451866</v>
       </c>
       <c r="F15">
-        <v>0.000908910261447357</v>
+        <v>0.0007199586310698626</v>
       </c>
       <c r="G15">
-        <v>0.01045246800664461</v>
+        <v>0.006062350857029151</v>
       </c>
       <c r="H15">
-        <v>0.008323704499570532</v>
+        <v>0.004883175061039501</v>
       </c>
       <c r="I15">
-        <v>209</v>
+        <v>403</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>tags=67%, list=22%, signal=53%</t>
+          <t>tags=53%, list=42%, signal=42%</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>51230/11091/10856/4297/23269/9070/3054/6045/5929/1876/4149/6872</t>
+          <t>2099/55929/3215/2077/4901/9575/7706/2122/64344/7750/79692/5948/90993/3661/57591/3651/2521/3096/571/147912/51523/9839/6657/1523/367/9611/5324/324/4298/9112/602/7026/4286/7541/57178/6777/11278/7775/26523/7027/54617/3183/8473/49854/4683/408/26205/3609/81608/3662/7157/9188/7538/51230/3110/1820/8314/7022/5885/8243/10856/3660/7728/860/5468/10725/7520/2353/22882/7494/5970/4772/4205/6945/6935/5093/9314/4605/2308/9324/7030/4089/7421/6774/1316/8932/11279/905/2313/4297/5977/2033/4790/140690/1021/9126/25836/10274/3659/3297/196/4086/5914/2908/1387/6670/5371/4090/53335/5925/3065/5241/4686/1022/4780/1027/4851/6772/8805/3091/4602/54973/2078/4088/4899/4601/9682/687/6671/5978/5460/10765/7469</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GO:0044665</t>
+          <t>GO:1990234</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MLL1/2 complex</t>
+          <t>transferase complex</t>
         </is>
       </c>
       <c r="C16">
-        <v>19</v>
+        <v>81</v>
       </c>
       <c r="D16">
-        <v>-0.459490693037087</v>
+        <v>-0.2080019315079769</v>
       </c>
       <c r="E16">
-        <v>-2.445867136667184</v>
+        <v>-2.275943121975419</v>
       </c>
       <c r="F16">
-        <v>0.0004544790395210988</v>
+        <v>0.001052086835603785</v>
       </c>
       <c r="G16">
-        <v>0.005807232171658486</v>
+        <v>0.00806599907296235</v>
       </c>
       <c r="H16">
-        <v>0.004624523560039251</v>
+        <v>0.006497097651447935</v>
       </c>
       <c r="I16">
         <v>209</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>tags=68%, list=22%, signal=55%</t>
+          <t>tags=43%, list=22%, signal=37%</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>51230/11091/10856/4297/23269/9070/3054/6045/5929/9757/1876/4149/6872</t>
+          <t>83860/7520/9968/2145/2648/5469/8085/3066/23512/905/4297/9070/2146/2033/672/1021/23269/6045/5929/3054/1387/51341/5925/1022/1027/2962/2959/1024/9757/1876/54880/4149/1025/6872/6908</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>GO:0005737</t>
+          <t>GO:0035770</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>cytoplasm</t>
+          <t>ribonucleoprotein granule</t>
         </is>
       </c>
       <c r="C17">
-        <v>424</v>
+        <v>13</v>
       </c>
       <c r="D17">
-        <v>-0.1246803923357143</v>
+        <v>-0.4844803928852141</v>
       </c>
       <c r="E17">
-        <v>-2.48921492355484</v>
+        <v>-2.183647059039652</v>
       </c>
       <c r="F17">
-        <v>0.0002086378167135866</v>
+        <v>0.002258622275661551</v>
       </c>
       <c r="G17">
-        <v>0.002999168615257808</v>
+        <v>0.01623384760631739</v>
       </c>
       <c r="H17">
-        <v>0.002388353954484479</v>
+        <v>0.01307623422751424</v>
       </c>
       <c r="I17">
-        <v>347</v>
+        <v>425</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>tags=44%, list=36%, signal=50%</t>
+          <t>tags=92%, list=44%, signal=52%</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>3096/7750/57178/2077/5316/1051/367/324/6777/7027/8473/3215/7026/571/6426/7775/6714/3190/408/4298/11016/3146/55553/84232/11278/2521/4286/5324/9112/4683/26205/9188/10445/7913/7538/7706/49854/3609/1105/8626/5468/8148/6495/26523/1820/2648/3170/7157/7728/8314/860/4772/55818/81608/3660/4609/84662/4205/3662/23309/22882/2353/7494/1877/64332/51548/7520/7541/3110/2002/6945/57504/10614/221937/51230/10725/8243/10856/3183/5970/6929/23435/9889/5093/121340/7004/7421/7764/6935/5885/8932/4089/4605/1316/7030/54617/6497/9314/672/2308/7022/6722/1487/3659/9324/1021/3297/3172/7391/2313/5977/11279/3066/196/4297/25836/6909/5914/6774/4790/905/4086/55726/4778/10274/2033/8553/9126/6670/4090/2624/3054/5371/1022/55734/10691/80319/140690/1027/4851/1387/4654/2908/1390/604/4760/4686/6045/5925/5451/53335/4780/4094/3516/5241/4602/3065/6772/1958/6938/54973/4209/4088/3091/6599/2113/8805/51341/688/10215/4899/687/1874/2078/6671/9682/4601/405/10765/7469/5978/1025/1869/5460/6667/6046/6908</t>
+          <t>2553/3191/9575/7706/3190/26523/7538/64332/23435/5093/3297/1025</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GO:1902494</t>
+          <t>GO:0000791</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>catalytic complex</t>
+          <t>euchromatin</t>
         </is>
       </c>
       <c r="C18">
-        <v>148</v>
+        <v>23</v>
       </c>
       <c r="D18">
-        <v>-0.1758842561870777</v>
+        <v>-0.3529286417726635</v>
       </c>
       <c r="E18">
-        <v>-2.582359194989498</v>
+        <v>-2.164062719573596</v>
       </c>
       <c r="F18">
-        <v>0.0001711296282795975</v>
+        <v>0.003416416284439833</v>
       </c>
       <c r="G18">
-        <v>0.002811415321736244</v>
+        <v>0.02311105133591651</v>
       </c>
       <c r="H18">
-        <v>0.002238838745913531</v>
+        <v>0.01861576675112726</v>
       </c>
       <c r="I18">
-        <v>399</v>
+        <v>226</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>tags=58%, list=41%, signal=40%</t>
+          <t>tags=61%, list=24%, signal=48%</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1499/9611/6597/1386/7307/2122/55249/23468/6907/55929/57459/324/23135/8535/8473/6426/221037/3190/9219/9112/9188/56970/10445/22976/7913/2145/26523/10042/2648/55818/9968/23309/79718/7520/57504/51230/11091/10856/3183/5469/8085/7764/83860/8932/54617/672/23512/1021/8289/5977/3066/4297/23269/6598/23186/905/2146/9070/2033/3054/1022/1027/1387/64919/23028/6045/5925/53335/2962/2959/3065/5929/6599/51341/1024/65980/9757/196528/1876/25942/54880/1025/4149/7528/6908/6872</t>
+          <t>10856/6929/9314/9070/3297/4654/6045/27125/3725/8805/3091/1385/6667/6908</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>GO:0005829</t>
+          <t>GO:1902562</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>cytosol</t>
+          <t>H4 histone acetyltransferase complex</t>
         </is>
       </c>
       <c r="C19">
-        <v>249</v>
+        <v>11</v>
       </c>
       <c r="D19">
-        <v>-0.1490103202958628</v>
+        <v>-0.4773773641734039</v>
       </c>
       <c r="E19">
-        <v>-2.617070737131445</v>
+        <v>-1.980441390796278</v>
       </c>
       <c r="F19">
-        <v>0.000170351711650198</v>
+        <v>0.005835590947991037</v>
       </c>
       <c r="G19">
-        <v>0.002811415321736244</v>
+        <v>0.03532068205362996</v>
       </c>
       <c r="H19">
-        <v>0.002238838745913531</v>
+        <v>0.02845052650544107</v>
       </c>
       <c r="I19">
-        <v>433</v>
+        <v>417</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>tags=57%, list=45%, signal=43%</t>
+          <t>tags=91%, list=43%, signal=52%</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>9575/79753/79692/90850/147912/2034/51523/90993/1523/2099/5948/3651/1499/9611/55893/10735/7025/84307/2122/6657/8531/4901/602/57591/9839/64344/55929/3096/7750/57178/2077/367/324/6777/7027/8473/3215/7026/571/7775/6714/408/4298/84232/11278/2521/4286/5324/9112/4683/26205/9188/7538/7706/49854/3609/5468/26523/1820/7157/7728/8314/860/4772/81608/3660/4205/3662/22882/2353/7494/7520/7541/3110/6945/51230/10725/8243/10856/3183/5970/5093/7421/6935/5885/8932/4089/4605/1316/7030/54617/9314/2308/7022/3659/9324/1021/3297/2313/5977/11279/196/4297/25836/5914/6774/4790/905/4086/10274/2033/9126/6670/4090/5371/1022/140690/1027/4851/1387/2908/4686/5925/53335/4780/5241/4602/3065/6772/54973/4088/3091/8805/4899/687/2078/6671/9682/4601/10765/7469/5978/5460</t>
+          <t>57634/55929/84148/1386/10445/8473/11091/51230/10856/3054</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GO:0090575</t>
+          <t>GO:0036464</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>RNA polymerase II transcription regulator complex</t>
+          <t>cytoplasmic ribonucleoprotein granule</t>
         </is>
       </c>
       <c r="C20">
-        <v>122</v>
+        <v>11</v>
       </c>
       <c r="D20">
-        <v>-0.2006495082610016</v>
+        <v>-0.4773445732349842</v>
       </c>
       <c r="E20">
-        <v>-2.727381413845893</v>
+        <v>-1.980305354744795</v>
       </c>
       <c r="F20">
-        <v>0.0001428524309473976</v>
+        <v>0.005835590947991037</v>
       </c>
       <c r="G20">
-        <v>0.002811415321736244</v>
+        <v>0.03532068205362996</v>
       </c>
       <c r="H20">
-        <v>0.002238838745913531</v>
+        <v>0.02845052650544107</v>
       </c>
       <c r="I20">
-        <v>245</v>
+        <v>508</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>tags=45%, list=25%, signal=38%</t>
+          <t>tags=100%, list=53%, signal=48%</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>4609/8861/1406/2353/7494/1050/4802/10589/6929/7421/5469/1052/83860/4089/466/5994/7029/467/4801/5914/6774/4086/4778/6934/4090/1022/4841/1390/4760/5925/5451/4780/4094/2962/2959/4602/3727/6772/6938/3725/4088/4800/3091/1874/9441/865/4601/1876/861/405/1869/4149/1385/6908/6872</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>GO:0005667</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>transcription regulator complex</t>
-        </is>
-      </c>
-      <c r="C21">
-        <v>235</v>
-      </c>
-      <c r="D21">
-        <v>-0.1577912648076182</v>
-      </c>
-      <c r="E21">
-        <v>-2.739366750676907</v>
-      </c>
-      <c r="F21">
-        <v>3.339003307208809E-05</v>
-      </c>
-      <c r="G21">
-        <v>0.0009599634508225327</v>
-      </c>
-      <c r="H21">
-        <v>0.0007644560203346485</v>
-      </c>
-      <c r="I21">
-        <v>275</v>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>tags=42%, list=29%, signal=40%</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>5468/56980/6495/2648/7157/5993/132660/860/4772/4609/2623/4205/8861/79718/1406/2353/7494/6886/6928/1050/57504/4802/10589/10725/5970/6929/7004/7421/5469/1052/83860/8932/4089/466/5994/6497/9314/7029/1487/7391/3066/196/467/4801/6909/5914/6774/4790/23186/4086/4778/2033/6934/6670/4090/2624/1022/1387/4654/4841/10481/23028/1390/4760/5925/5451/4780/4094/2962/8328/3516/2959/4602/3065/3727/6772/6938/3725/4088/4800/3091/688/1874/9441/865/4601/1876/861/405/25942/5978/1869/5460/4149/7528/6667/1385/6908/6872</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>GO:0140513</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>nuclear protein-containing complex</t>
-        </is>
-      </c>
-      <c r="C22">
-        <v>287</v>
-      </c>
-      <c r="D22">
-        <v>-0.1766257608121525</v>
-      </c>
-      <c r="E22">
-        <v>-3.248530395263305</v>
-      </c>
-      <c r="F22">
-        <v>4.097012559283651E-07</v>
-      </c>
-      <c r="G22">
-        <v>1.570521481058733E-05</v>
-      </c>
-      <c r="H22">
-        <v>1.250666991781325E-05</v>
-      </c>
-      <c r="I22">
-        <v>342</v>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>tags=49%, list=35%, signal=45%</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>1051/23135/8535/6777/7027/8473/571/6426/221037/3190/4298/11016/9219/9112/4683/9188/56970/10445/22976/7913/2626/2145/80816/5468/10042/2648/5993/132660/8314/55818/81608/9968/4609/8861/23309/79718/1406/2353/7494/7520/1050/57504/10614/51230/4802/11091/10589/10856/3183/84844/5970/6929/22936/7421/5469/8085/7764/1052/83860/8932/4089/4605/466/5994/54617/672/7029/23512/8289/5977/51497/3066/196/4297/467/4801/25836/23269/5914/6774/6598/4790/23186/905/4086/55726/2146/4778/9070/6934/4090/3054/1022/64919/27125/4841/1390/4760/6045/5925/5451/53335/4780/4094/2962/2959/4602/3065/3727/6772/6938/54973/3725/4088/5929/4800/3091/6599/51341/1024/65980/9757/1874/9441/196528/865/4601/1876/861/405/25942/7936/6829/7469/54880/1025/1869/4149/7528/1385/6908/6872</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>GO:0000785</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>chromatin</t>
-        </is>
-      </c>
-      <c r="C23">
-        <v>476</v>
-      </c>
-      <c r="D23">
-        <v>-0.1683054408510895</v>
-      </c>
-      <c r="E23">
-        <v>-3.337089085658244</v>
-      </c>
-      <c r="F23">
-        <v>2.203374326208636E-07</v>
-      </c>
-      <c r="G23">
-        <v>1.266940237569966E-05</v>
-      </c>
-      <c r="H23">
-        <v>1.008913507263954E-05</v>
-      </c>
-      <c r="I23">
-        <v>426</v>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>tags=54%, list=44%, signal=59%</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>147912/6662/8819/6932/2034/1879/10472/10155/90993/84913/1523/2099/60436/2101/3651/2118/3726/1499/23394/9611/23272/10735/7080/128209/2355/6597/1386/83855/5090/55249/6657/5309/7392/4901/2627/23468/9839/7020/7552/64344/55929/57459/57178/2077/5316/1051/367/6777/3169/7027/5927/8473/3215/571/221037/79977/3190/408/11016/55553/10608/11278/4286/9219/9112/28999/26205/9188/6688/56970/3222/10445/7913/116113/2626/23030/11244/2145/2115/1105/8626/5468/56980/6495/10042/2648/3170/7157/5993/10919/7182/860/4772/55818/7544/3660/4609/2623/4205/3662/8861/23309/22882/55145/1406/2353/51548/6886/6928/3110/1050/2002/6945/57504/221937/51230/4802/11091/10725/3200/10856/3183/30009/5970/6929/23435/9889/121340/7004/7421/5469/1052/6935/5885/8932/4089/64843/1316/466/7030/54617/23476/9314/93986/7543/2308/7022/23081/7029/26959/23512/79923/6722/3659/9324/3297/3172/8289/7391/2313/5977/6096/11279/3066/196/7071/389058/2551/467/4801/25836/6909/546/23269/5914/4335/6774/6598/4790/27086/4086/2146/4778/9070/10274/2033/8553/6934/9126/10951/6670/4090/3054/10691/2625/1387/64919/27125/4654/5079/2908/10481/23028/1390/4760/6045/5925/5451/53335/4780/4094/3516/5241/3065/3727/6772/10661/1958/6938/3725/4209/4088/4800/3091/6599/2113/8805/688/65980/1106/10215/687/8019/1874/2078/6671/196528/9682/4601/1876/861/405/25942/4613/7936/1997/10765/6668/1869/4149/7528/6667/1385/6046/6908/6872</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>GO:0032991</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>protein-containing complex</t>
-        </is>
-      </c>
-      <c r="C24">
-        <v>429</v>
-      </c>
-      <c r="D24">
-        <v>-0.1730849465578376</v>
-      </c>
-      <c r="E24">
-        <v>-3.464610230308045</v>
-      </c>
-      <c r="F24">
-        <v>6.240493959311298E-08</v>
-      </c>
-      <c r="G24">
-        <v>7.176568053207993E-06</v>
-      </c>
-      <c r="H24">
-        <v>5.714978678527189E-06</v>
-      </c>
-      <c r="I24">
-        <v>343</v>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>tags=46%, list=36%, signal=54%</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>5316/1051/367/324/23135/8535/6777/7027/5927/8473/571/6426/221037/3190/4298/11016/3146/4286/9219/29781/9112/4683/9188/6688/56970/10445/22976/7913/7538/2626/2145/80816/3609/8626/5468/56980/6495/26523/10042/2648/7157/5993/132660/8314/860/4772/55818/657/81608/9968/4609/2623/4205/3662/8861/23309/79718/1406/2353/7494/7520/6886/6928/1050/57504/10614/51230/4802/11091/10589/10725/8243/10856/3183/84844/5970/6929/5093/22936/7004/7421/5469/8085/7764/1052/83860/5885/8932/4089/4605/466/5994/54617/6497/9314/672/9584/7029/23512/1487/1021/3297/8289/7391/5977/51497/3066/196/4297/467/4801/25836/6909/23269/5914/6774/6598/4790/23186/905/4086/55726/2146/4778/9070/10274/2033/6934/9126/6670/4090/2624/3054/1022/1027/4851/1387/64919/27125/4654/4841/2908/10481/23028/1390/4760/4686/6045/5925/5451/53335/4780/92906/4094/2962/8328/3516/2959/4602/3065/3727/6772/6938/54973/3725/4088/5929/4800/3091/6599/51341/1024/688/65980/9757/1874/2078/9441/196528/865/4601/1876/861/405/25942/7936/6829/7469/54880/5978/1025/1869/5460/4149/7528/6667/1385/6908/6872</t>
+          <t>2553/9575/7706/3190/26523/7538/64332/23435/5093/1025</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1236,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1471,473 +1299,387 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GO:0000791</t>
+          <t>GO:1902494</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>euchromatin</t>
+          <t>catalytic complex</t>
         </is>
       </c>
       <c r="C2">
-        <v>23</v>
+        <v>148</v>
       </c>
       <c r="D2">
-        <v>-0.3273262666103552</v>
+        <v>-0.1970029984061649</v>
       </c>
       <c r="E2">
-        <v>-1.888521650937372</v>
+        <v>-2.676213128005946</v>
       </c>
       <c r="F2">
-        <v>0.006286580303872253</v>
+        <v>1.886312926183766E-05</v>
       </c>
       <c r="G2">
-        <v>0.07229567349453091</v>
+        <v>0.002169259865111331</v>
       </c>
       <c r="H2">
-        <v>0.06286580303872254</v>
+        <v>0.00186645700064499</v>
       </c>
       <c r="I2">
-        <v>223</v>
+        <v>559</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>tags=57%, list=23%, signal=45%</t>
+          <t>tags=76%, list=58%, signal=37%</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>10856/6929/9314/27125/9070/6045/3725/3091/4654/6908/6667/1385/8805</t>
+          <t>55249/8607/53615/8850/57634/23054/5591/1457/7307/22823/6760/4221/84759/7520/3187/8473/10013/3720/2122/5928/9219/9611/9188/8467/7913/23492/55696/57680/57492/7703/6604/5926/1499/2145/23309/1655/6907/29117/324/672/8819/23186/6426/79718/57504/10445/221037/56970/23269/22976/63925/2146/57459/51230/5977/10856/3066/10042/1021/8932/8085/23512/1022/83860/55929/64919/3190/11143/53335/2033/2959/7764/905/9070/2962/54815/55818/5925/3054/9112/1387/65980/26523/6597/4297/5469/23028/8535/1027/6908/6598/23135/1024/6045/8289/54617/1876/26147/11091/6599/9757/5929/3183/196528/7528/51341/3065/25942/4149/6872/54880/1025</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GO:0044665</t>
+          <t>GO:0140513</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MLL1/2 complex</t>
+          <t>nuclear protein-containing complex</t>
         </is>
       </c>
       <c r="C3">
-        <v>19</v>
+        <v>287</v>
       </c>
       <c r="D3">
-        <v>-0.3788702584558448</v>
+        <v>-0.1520177077494346</v>
       </c>
       <c r="E3">
-        <v>-1.977671227502474</v>
+        <v>-2.603467793731186</v>
       </c>
       <c r="F3">
-        <v>0.005763764541390992</v>
+        <v>6.447382080381014E-05</v>
       </c>
       <c r="G3">
-        <v>0.07229567349453091</v>
+        <v>0.003707244696219083</v>
       </c>
       <c r="H3">
-        <v>0.06286580303872254</v>
+        <v>0.003189757450293765</v>
       </c>
       <c r="I3">
-        <v>287</v>
+        <v>488</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>tags=68%, list=30%, signal=49%</t>
+          <t>tags=62%, list=51%, signal=44%</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>10445/51230/10856/9070/3054/6045/4297/1876/11091/9757/5929/4149/6872</t>
+          <t>84759/5971/8314/7494/7520/3187/8473/2353/10013/2355/5993/6777/3720/4298/2122/7068/4087/5928/9219/9611/9188/4683/8467/7913/7027/55120/1406/23492/2309/55696/57680/57492/7703/6604/8861/5926/1499/2145/23309/1655/6907/29117/23429/1051/672/11335/7421/8819/23186/6426/80816/79718/7090/57504/10445/2626/22936/4094/5468/221037/11016/1050/10155/4089/56970/23269/6256/6932/4802/22976/196/63925/2146/5970/57459/4780/571/4801/51230/5977/10856/3066/4090/10042/8932/8085/23512/6934/81608/1022/83860/84844/4800/4778/55929/4760/64919/3190/11143/27125/53335/25836/3727/2959/55726/5994/51497/7764/905/9070/4086/2962/10589/5914/54815/55818/466/5925/6938/6929/4602/3054/132660/5451/9112/1390/6772/65980/6774/6597/4297/6829/467/5469/7469/54973/8535/4609/6908/6598/23135/1024/4841/6045/9441/4790/3725/1874/8289/4605/54617/1052/1876/3091/26147/405/7029/4601/11091/6599/9757/7936/5929/4088/865/1385/3183/10614/861/196528/7528/51341/1869/3065/25942/4149/6872/54880/1025</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GO:0099080</t>
+          <t>GO:0070603</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>supramolecular complex</t>
+          <t>SWI/SNF superfamily-type complex</t>
         </is>
       </c>
       <c r="C4">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="D4">
-        <v>-0.2727039280104081</v>
+        <v>-0.2653120604819508</v>
       </c>
       <c r="E4">
-        <v>-2.01699823946486</v>
+        <v>-2.114545382237919</v>
       </c>
       <c r="F4">
-        <v>0.007398377653571694</v>
+        <v>0.001969038386022641</v>
       </c>
       <c r="G4">
-        <v>0.07734667546915863</v>
+        <v>0.05660985359815092</v>
       </c>
       <c r="H4">
-        <v>0.06725797866883358</v>
+        <v>0.04870779165424428</v>
       </c>
       <c r="I4">
-        <v>600</v>
+        <v>559</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>tags=89%, list=62%, signal=35%</t>
+          <t>tags=84%, list=58%, signal=37%</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>7756/7150/8850/7538/6605/2553/7913/23468/3191/10013/1499/324/3297/29117/5093/64332/6714/23435/9112/2959/8243/3190/26523/6597/92822/6598/54617/4654/6599/196528/25942/7706/1025</t>
+          <t>55249/8607/53615/57634/6760/5928/9219/9188/8467/7913/57492/6604/29117/57504/10445/57459/5977/10856/3066/10042/8932/23512/55929/64919/53335/54815/5925/9112/65980/6597/6598/8289/54617/6599/196528/7528/3065</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GO:0070603</t>
+          <t>GO:1904949</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SWI/SNF superfamily-type complex</t>
+          <t>ATPase complex</t>
         </is>
       </c>
       <c r="C5">
         <v>44</v>
       </c>
       <c r="D5">
-        <v>-0.2554767391221578</v>
+        <v>-0.2653120604819508</v>
       </c>
       <c r="E5">
-        <v>-2.024458466288952</v>
+        <v>-2.114545382237919</v>
       </c>
       <c r="F5">
-        <v>0.004368951233579065</v>
+        <v>0.001969038386022641</v>
       </c>
       <c r="G5">
-        <v>0.07229567349453091</v>
+        <v>0.05660985359815092</v>
       </c>
       <c r="H5">
-        <v>0.06286580303872254</v>
+        <v>0.04870779165424428</v>
       </c>
       <c r="I5">
-        <v>593</v>
+        <v>559</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>tags=86%, list=62%, signal=35%</t>
+          <t>tags=84%, list=58%, signal=37%</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>9219/29998/55249/8607/6604/9188/5928/6605/7913/53615/6760/57504/8932/57492/8467/29117/10445/23512/57459/3066/10856/64919/10042/9112/53335/54815/55929/5977/5925/6597/65980/6598/8289/54617/6599/196528/7528/3065</t>
+          <t>55249/8607/53615/57634/6760/5928/9219/9188/8467/7913/57492/6604/29117/57504/10445/57459/5977/10856/3066/10042/8932/23512/55929/64919/53335/54815/5925/9112/65980/6597/6598/8289/54617/6599/196528/7528/3065</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GO:1904949</t>
+          <t>GO:0000775</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ATPase complex</t>
+          <t>chromosome, centromeric region</t>
         </is>
       </c>
       <c r="C6">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="D6">
-        <v>-0.2554767391221578</v>
+        <v>-0.3005634559869776</v>
       </c>
       <c r="E6">
-        <v>-2.024458466288952</v>
+        <v>-2.170364057660885</v>
       </c>
       <c r="F6">
-        <v>0.004368951233579065</v>
+        <v>0.002520433072871786</v>
       </c>
       <c r="G6">
-        <v>0.07229567349453091</v>
+        <v>0.05796996067605108</v>
       </c>
       <c r="H6">
-        <v>0.06286580303872254</v>
+        <v>0.04987804396841009</v>
       </c>
       <c r="I6">
-        <v>593</v>
+        <v>378</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>tags=86%, list=62%, signal=35%</t>
+          <t>tags=69%, list=39%, signal=44%</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>9219/29998/55249/8607/6604/9188/5928/6605/7913/53615/6760/57504/8932/57492/8467/29117/10445/23512/57459/3066/10856/64919/10042/9112/53335/54815/55929/5977/5925/6597/65980/6598/8289/54617/6599/196528/7528/3065</t>
+          <t>29117/324/1051/11335/10664/2146/3297/9126/10951/8243/11143/546/2959/51548/5885/10735/92822/6597/10274/6598/6599/23081/196528/9682/25942</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GO:0034708</t>
+          <t>GO:0000791</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>methyltransferase complex</t>
+          <t>euchromatin</t>
         </is>
       </c>
       <c r="C7">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="D7">
-        <v>-0.2841857031353661</v>
+        <v>-0.3447634991841628</v>
       </c>
       <c r="E7">
-        <v>-2.051016497196311</v>
+        <v>-2.077592823947477</v>
       </c>
       <c r="F7">
-        <v>0.005877916189770061</v>
+        <v>0.005115155712782556</v>
       </c>
       <c r="G7">
-        <v>0.07229567349453091</v>
+        <v>0.08096398566883629</v>
       </c>
       <c r="H7">
-        <v>0.06286580303872254</v>
+        <v>0.06966237668531454</v>
       </c>
       <c r="I7">
-        <v>314</v>
+        <v>414</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>tags=61%, list=33%, signal=43%</t>
+          <t>tags=78%, list=43%, signal=46%</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>22976/2146/10445/63925/3720/51230/23512/8085/3066/10856/9070/3054/26147/23135/6045/4297/1876/11091/9757/5929/4149/6872</t>
+          <t>2099/1499/11335/10155/3297/10856/27125/9314/9070/6929/6908/6045/4654/3725/6667/3091/1385/8805</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GO:0035097</t>
+          <t>GO:0099080</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>histone methyltransferase complex</t>
+          <t>supramolecular complex</t>
         </is>
       </c>
       <c r="C8">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D8">
-        <v>-0.2841857031353661</v>
+        <v>-0.2752686722340424</v>
       </c>
       <c r="E8">
-        <v>-2.051016497196311</v>
+        <v>-2.025919429286129</v>
       </c>
       <c r="F8">
-        <v>0.005877916189770061</v>
+        <v>0.005357045904420018</v>
       </c>
       <c r="G8">
-        <v>0.07229567349453091</v>
+        <v>0.08096398566883629</v>
       </c>
       <c r="H8">
-        <v>0.06286580303872254</v>
+        <v>0.06966237668531454</v>
       </c>
       <c r="I8">
-        <v>314</v>
+        <v>437</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>tags=61%, list=33%, signal=43%</t>
+          <t>tags=73%, list=46%, signal=41%</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>22976/2146/10445/63925/3720/51230/23512/8085/3066/10856/9070/3054/26147/23135/6045/4297/1876/11091/9757/5929/4149/6872</t>
+          <t>7913/7538/2553/3191/1499/29117/324/6714/64332/3297/23435/5093/8243/3190/2959/92822/9112/26523/6597/6598/4654/54617/6599/7706/196528/25942/1025</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GO:1990234</t>
+          <t>GO:0044665</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>transferase complex</t>
+          <t>MLL1/2 complex</t>
         </is>
       </c>
       <c r="C9">
-        <v>81</v>
+        <v>19</v>
       </c>
       <c r="D9">
-        <v>-0.1999975176139968</v>
+        <v>-0.3778480765222647</v>
       </c>
       <c r="E9">
-        <v>-2.121476992659138</v>
+        <v>-2.012584222857691</v>
       </c>
       <c r="F9">
-        <v>0.003524882048770449</v>
+        <v>0.005632277263919046</v>
       </c>
       <c r="G9">
-        <v>0.07229567349453091</v>
+        <v>0.08096398566883629</v>
       </c>
       <c r="H9">
-        <v>0.06286580303872254</v>
+        <v>0.06966237668531454</v>
       </c>
       <c r="I9">
-        <v>287</v>
+        <v>341</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>tags=49%, list=30%, signal=38%</t>
+          <t>tags=74%, list=36%, signal=48%</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>10445/56970/1022/63925/3720/51230/23512/1021/8085/3066/10856/5469/2959/55929/2033/83860/905/2962/1387/9070/5925/3054/26147/23135/1027/6045/11143/4297/1024/6908/1876/11091/9757/5929/8535/4149/51341/1025/6872/54880</t>
+          <t>10445/23269/51230/10856/9070/3054/4297/6045/1876/11091/9757/5929/4149/6872</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GO:0140513</t>
+          <t>GO:1990234</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>nuclear protein-containing complex</t>
+          <t>transferase complex</t>
         </is>
       </c>
       <c r="C10">
-        <v>287</v>
+        <v>81</v>
       </c>
       <c r="D10">
-        <v>-0.1247859333879007</v>
+        <v>-0.1801795030985247</v>
       </c>
       <c r="E10">
-        <v>-2.204506191682019</v>
+        <v>-1.92434054868048</v>
       </c>
       <c r="F10">
-        <v>0.001374587986442749</v>
+        <v>0.007397614878304447</v>
       </c>
       <c r="G10">
-        <v>0.07229567349453091</v>
+        <v>0.09452507900055683</v>
       </c>
       <c r="H10">
-        <v>0.06286580303872254</v>
+        <v>0.08133050275562784</v>
       </c>
       <c r="I10">
-        <v>407</v>
+        <v>316</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>tags=52%, list=42%, signal=43%</t>
+          <t>tags=51%, list=33%, signal=37%</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>6426/55696/7421/8819/11016/22936/23269/7703/23429/6760/5926/80816/23186/1655/672/57504/8861/22823/2626/4087/8932/57492/10155/196/79718/4089/4094/8467/221037/55120/2309/4780/22976/11335/1050/29117/2146/5468/4802/10445/56970/5970/1022/63925/81608/4801/3720/51230/5451/6932/23512/4090/571/4760/57459/6256/51497/4800/8085/3066/5914/10856/7764/5469/64919/25836/10042/9112/6938/53335/54815/84844/6929/466/2959/5994/55929/1390/4778/5977/6934/55726/3727/83860/10589/27125/3190/905/2962/9070/4602/55818/5925/4086/3054/6597/26147/23135/6774/132660/467/7469/9441/6772/65980/6045/54973/4609/11143/6598/6829/4841/1874/4297/3725/405/4790/1024/3091/8289/54617/1052/6908/4601/1876/4605/7936/7029/4088/11091/865/6599/9757/5929/861/8535/1385/1869/10614/196528/7528/3183/25942/3065/4149/51341/1025/6872/54880</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>GO:0000775</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>chromosome, centromeric region</t>
-        </is>
-      </c>
-      <c r="C11">
-        <v>36</v>
-      </c>
-      <c r="D11">
-        <v>-0.3073793413913595</v>
-      </c>
-      <c r="E11">
-        <v>-2.218408924641497</v>
-      </c>
-      <c r="F11">
-        <v>0.002133366743201307</v>
-      </c>
-      <c r="G11">
-        <v>0.07229567349453091</v>
-      </c>
-      <c r="H11">
-        <v>0.06286580303872254</v>
-      </c>
-      <c r="I11">
-        <v>345</v>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>tags=67%, list=36%, signal=44%</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>10664/8467/11335/3297/29117/2146/10951/9126/546/2959/8243/5885/6597/10735/92822/10274/51548/11143/6598/23081/6599/9682/196528/25942</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>GO:1902494</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>catalytic complex</t>
-        </is>
-      </c>
-      <c r="C12">
-        <v>148</v>
-      </c>
-      <c r="D12">
-        <v>-0.1898163918062701</v>
-      </c>
-      <c r="E12">
-        <v>-2.60561578885221</v>
-      </c>
-      <c r="F12">
-        <v>0.0002479856035655127</v>
-      </c>
-      <c r="G12">
-        <v>0.02851834441003396</v>
-      </c>
-      <c r="H12">
-        <v>0.02479856035655127</v>
-      </c>
-      <c r="I12">
-        <v>593</v>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>tags=78%, list=62%, signal=36%</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>9219/29998/55249/8607/8473/5591/8850/6604/57680/1457/9188/58508/5928/51317/3187/6605/2145/7307/4221/7913/23468/7520/54623/10013/23492/84759/6907/23309/1499/9611/2122/53615/6426/55696/8819/23269/7703/6760/5926/23186/1655/672/57504/324/22823/8932/57492/79718/8467/221037/22976/29117/2146/10445/56970/1022/63925/3720/51230/23512/57459/1021/8085/3066/10856/7764/5469/64919/10042/9112/53335/54815/2959/55929/5977/2033/83860/3190/26523/905/2962/1387/9070/55818/5925/3054/6597/26147/23135/1027/65980/6045/23028/11143/6598/4297/1024/8289/54617/6908/1876/11091/6599/9757/5929/8535/196528/7528/3183/25942/3065/4149/51341/1025/6872/54880</t>
+          <t>56970/23269/22976/63925/2146/51230/10856/3066/1021/8085/23512/1022/83860/55929/11143/2033/2959/905/9070/2962/5925/3054/1387/4297/5469/8535/1027/6908/23135/1024/6045/1876/26147/11091/9757/5929/51341/4149/6872/54880/1025</t>
         </is>
       </c>
     </row>

</xml_diff>